<commit_message>
Rework: per-organization models with auto-training, honest forecasts (verdict, interval, budget window), currency support, real-data-calibrated generator
</commit_message>
<xml_diff>
--- a/db/generator/exports/sample_upload_1.xlsx
+++ b/db/generator/exports/sample_upload_1.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,1026 +446,1566 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>124449</t>
+          <t>541885</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2011</t>
+          <t>17243</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>926.1</t>
+          <t>334.52</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>719.12</t>
+          <t>998.99</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>161472</t>
+          <t>1123172</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2088</t>
+          <t>34115</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>926.11</t>
+          <t>664.06</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>787.69</t>
+          <t>1872.4</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>125948</t>
+          <t>1615774</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1918</t>
+          <t>46702</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>925.76</t>
+          <t>955.76</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>798.08</t>
+          <t>1751.14</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>148055</t>
+          <t>1666602</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2091</t>
+          <t>48315</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>926.03</t>
+          <t>999.07</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>864.52</t>
+          <t>2649.42</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>150103</t>
+          <t>1585421</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2059</t>
+          <t>50719</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>926.1</t>
+          <t>1013.24</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>637.59</t>
+          <t>2424.36</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>125961</t>
+          <t>1685806</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>1866</t>
+          <t>48526</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>925.95</t>
+          <t>987.74</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>570.76</t>
+          <t>1845.57</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>149526</t>
+          <t>1576638</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2117</t>
+          <t>49787</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>926.03</t>
+          <t>1011.6</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>643.86</t>
+          <t>2012.7</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>137967</t>
+          <t>1623424</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2060</t>
+          <t>52167</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>926.1</t>
+          <t>1055.93</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>820.66</t>
+          <t>2559.87</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>161895</t>
+          <t>1443840</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2088</t>
+          <t>48336</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>925.93</t>
+          <t>967.37</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>954.73</t>
+          <t>2165.35</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>138333</t>
+          <t>1863929</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2027</t>
+          <t>55446</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>926.13</t>
+          <t>1016.62</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>665.61</t>
+          <t>2097.75</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>144498</t>
+          <t>1596475</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2064</t>
+          <t>48772</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>926.09</t>
+          <t>953.21</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>738.14</t>
+          <t>2543.63</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>162399</t>
+          <t>1817628</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2254</t>
+          <t>52283</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>926.06</t>
+          <t>997.69</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>636.36</t>
+          <t>1799.88</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>164910</t>
+          <t>2019482</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2296</t>
+          <t>57524</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>926.06</t>
+          <t>1038.52</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>582.89</t>
+          <t>1857.81</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>133799</t>
+          <t>1470242</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>1992</t>
+          <t>48184</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>925.74</t>
+          <t>980.36</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>689.85</t>
+          <t>2975.16</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>139463</t>
+          <t>1632296</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>45798</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>926.12</t>
+          <t>985.2</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>774.98</t>
+          <t>2393.6</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>152554</t>
+          <t>1437446</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2014</t>
+          <t>47839</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>925.96</t>
+          <t>975.75</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>747.43</t>
+          <t>2308.86</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>142718</t>
+          <t>1761981</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2004</t>
+          <t>49459</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>926.18</t>
+          <t>1008.46</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>813.53</t>
+          <t>1917.72</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>156940</t>
+          <t>1653738</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2045</t>
+          <t>50669</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>925.95</t>
+          <t>988.4</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>757.32</t>
+          <t>2297.1</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>165888</t>
+          <t>1629456</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2259</t>
+          <t>48329</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>925.95</t>
+          <t>954.41</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>801.04</t>
+          <t>2289.47</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>150199</t>
+          <t>1689446</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2336</t>
+          <t>50243</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>926.0</t>
+          <t>976.84</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>750.87</t>
+          <t>2010.05</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>153699</t>
+          <t>1645069</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2168</t>
+          <t>52899</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>925.78</t>
+          <t>1023.04</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>789.85</t>
+          <t>2831.79</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>153172</t>
+          <t>1479019</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1951</t>
+          <t>48761</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>926.0</t>
+          <t>976.39</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>844.34</t>
+          <t>2514.99</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>157166</t>
+          <t>1641479</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2196</t>
+          <t>49872</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>925.93</t>
+          <t>982.64</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>794.38</t>
+          <t>1888.95</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>134605</t>
+          <t>1739271</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>50947</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>926.02</t>
+          <t>1020.43</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>869.53</t>
+          <t>2647.07</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>144660</t>
+          <t>1718529</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2119</t>
+          <t>52384</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>925.82</t>
+          <t>1052.02</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>787.4</t>
+          <t>3071.65</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>163722</t>
+          <t>1870951</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2217</t>
+          <t>54750</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>925.77</t>
+          <t>1011.61</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>708.35</t>
+          <t>2292.54</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>168703</t>
+          <t>1476414</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2255</t>
+          <t>46706</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>926.1</t>
+          <t>968.21</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>658.58</t>
+          <t>2420.36</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>141109</t>
+          <t>1459270</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2058</t>
+          <t>46373</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>926.18</t>
+          <t>970.29</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>683.91</t>
+          <t>2626.03</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>146588</t>
+          <t>1832225</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2099</t>
+          <t>51401</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>925.97</t>
+          <t>1008.98</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>898.36</t>
+          <t>1862.08</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>151340</t>
+          <t>1443044</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2065</t>
+          <t>48477</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>925.93</t>
+          <t>1010.47</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>784.46</t>
+          <t>2561.53</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>167637</t>
+          <t>1591180</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2284</t>
+          <t>47684</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>925.99</t>
+          <t>971.44</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>820.6</t>
+          <t>2080.36</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>163380</t>
+          <t>1481793</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2132</t>
+          <t>47585</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>925.95</t>
+          <t>999.23</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>651.33</t>
+          <t>2216.34</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>151778</t>
+          <t>1760955</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2030</t>
+          <t>52742</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>926.18</t>
+          <t>1030.85</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>636.88</t>
+          <t>2405.88</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>146015</t>
+          <t>1741697</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2067</t>
+          <t>49805</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>925.93</t>
+          <t>1002.04</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>456.66</t>
+          <t>1929.72</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>144243</t>
+          <t>1447266</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>1992</t>
+          <t>48318</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>925.97</t>
+          <t>976.7</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>500.42</t>
+          <t>2072.37</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>155281</t>
+          <t>1815761</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2029</t>
+          <t>49352</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>926.16</t>
+          <t>1004.6</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>736.03</t>
+          <t>2333.84</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>155739</t>
+          <t>1593534</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2170</t>
+          <t>48336</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>925.86</t>
+          <t>1028.47</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>751.16</t>
+          <t>1849.41</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>140790</t>
+          <t>1466392</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2049</t>
+          <t>43896</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>925.91</t>
+          <t>960.55</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>682.04</t>
+          <t>1851.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>1800049</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>54696</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>977.06</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>1599.21</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>1684425</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>51514</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>1038.89</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>1815.79</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>1696971</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>48316</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>997.03</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>1662.34</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>1622987</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>44364</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>973.14</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>1874.19</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>1942563</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>53690</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>999.28</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>1912.17</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>1485743</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>45716</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>944.15</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>1668.75</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>1818373</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>50536</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>1018.64</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>2127.54</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>1374727</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>44886</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>952.39</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>1496.43</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>1640658</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>51322</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>992.13</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>1622.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>1750779</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>52424</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>1058.99</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>1553.37</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>1765205</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>50066</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>982.14</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>1697.53</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>1581067</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>46873</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>966.96</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>1950.76</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>1508045</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>47960</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>974.95</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>2071.53</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>1565912</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>48726</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>999.32</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>1564.86</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>1954953</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>52684</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>1005.97</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>1669.21</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>1535672</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>47325</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>983.39</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>1420.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>1549159</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>48453</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>994.79</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>1347.63</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>1758149</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>50833</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>961.28</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>1950.44</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>1683589</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>50884</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>1013.49</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>1970.69</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>1899757</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>52233</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>983.68</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>1837.55</t>
         </is>
       </c>
     </row>

</xml_diff>